<commit_message>
improved clusters and bubble chart explanation
</commit_message>
<xml_diff>
--- a/data/output/authors_disambiguation_cluster_elastic.xlsx
+++ b/data/output/authors_disambiguation_cluster_elastic.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P101"/>
+  <dimension ref="A1:T101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,20 +479,40 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>co_authors</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>orcid_source</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>current_organization</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>cluster_id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>cluster_size</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>script</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>AKA</t>
         </is>
@@ -538,7 +558,11 @@
           <t>wang_y_0Tm4oOxx0UxjuLkqthOvk</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0000-0002-4871-5449</t>
+        </is>
+      </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
@@ -547,14 +571,34 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>['10.1103/physrevc.103.014902']</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>doi:10.1103/physrevc.103.014902</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>['Rutgers, The State University of New Jersey']</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>wang_y_0Tm4oOxx0UxjuLkqthOvk</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+      <c r="R2" t="n">
+        <v>4</v>
+      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -587,16 +631,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Gershtein, Y.</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>wang_y_2YfeZ8hOH15pQk1ejNpx5</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0000-0002-4871-5449</t>
+        </is>
+      </c>
       <c r="K3" t="n">
         <v>1</v>
       </c>
@@ -605,14 +657,34 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>wang_y_2YfeZ8hOH15pQk1ejNpx5</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+          <t>['10.1016/j.physletb.2019.06.021']</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>doi:10.1016/j.physletb.2019.06.021</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>['Rutgers, The State University of New Jersey']</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>wang_y_0Tm4oOxx0UxjuLkqthOvk</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>4</v>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -645,16 +717,24 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Gershtein, Y.</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>wang_y_5IW9GCctopP2loIerOuex</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0000-0002-4871-5449</t>
+        </is>
+      </c>
       <c r="K4" t="n">
         <v>3</v>
       </c>
@@ -663,18 +743,38 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>wang_y_5IW9GCctopP2loIerOuex</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>1</v>
+          <t>['10.1016/j.physletb.2021.136188', '10.1016/j.physletb.2021.136253']</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>doi:10.1016/j.physletb.2021.136188</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>['Rutgers, The State University of New Jersey', 'University of Wisconsin–Madison']</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>wang_y_0Tm4oOxx0UxjuLkqthOvk</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>4</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
           <t>{'source': "ctx._source.AKA ='wang_y_wIO6TkGmRtOgDDU2kRHYz'", 'lang': 'painless'}</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -707,16 +807,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Gershtein, Y.</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>wang_y_6hlWEOo-vPGbrklvdeRCF</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0000-0002-4871-5449</t>
+        </is>
+      </c>
       <c r="K5" t="n">
         <v>2</v>
       </c>
@@ -725,14 +833,34 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>wang_y_6hlWEOo-vPGbrklvdeRCF</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+          <t>['10.1103/physrevd.100.072007', '10.1103/physrevd.101.052010']</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>doi:10.1103/physrevd.100.072007</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>['Rutgers, The State University of New Jersey']</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>wang_y_0Tm4oOxx0UxjuLkqthOvk</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>4</v>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -783,14 +911,30 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
+          <t>['10.1140/epjc/s10052-018-6148-7']</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>['Texas A&amp;M University']</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>wang_y_1p5XpVjKs84NFU_WrIqCS</t>
         </is>
       </c>
-      <c r="N6" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+      <c r="R6" t="n">
+        <v>4</v>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -823,10 +967,14 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Pakhotin, Y.</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>wang_y_4_R2tEUxiB4RBBAKtj2FK</t>
@@ -841,14 +989,30 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>wang_y_4_R2tEUxiB4RBBAKtj2FK</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.98.092014']</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>['Texas A&amp;M University']</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>wang_y_1p5XpVjKs84NFU_WrIqCS</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>4</v>
+      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -881,10 +1045,14 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Pakhotin, Y.</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>wang_y_5woMN_aCLimFGR-kloTK0</t>
@@ -899,14 +1067,30 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>wang_y_5woMN_aCLimFGR-kloTK0</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>1</v>
+          <t>['10.1016/j.physletb.2019.01.005']</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>['Texas A&amp;M University']</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>wang_y_1p5XpVjKs84NFU_WrIqCS</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>4</v>
+      </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -939,10 +1123,14 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Pakhotin, Y.</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>wang_y_7EC9Xuu9rgPeQxv0-Q-20</t>
@@ -957,14 +1145,30 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>wang_y_7EC9Xuu9rgPeQxv0-Q-20</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep11(2018)152']</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>['Texas A&amp;M University']</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>wang_y_1p5XpVjKs84NFU_WrIqCS</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1006,7 +1210,11 @@
           <t>wang_y_5NkomzT3X1dvOMjcCQ8nP</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>0000-0003-3979-4330</t>
+        </is>
+      </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
@@ -1015,14 +1223,34 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
+          <t>['10.1103/physrevlett.131.041902']</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>doi:10.1103/physrevlett.131.041902</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>['Central China Normal University']</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
           <t>wang_y_5NkomzT3X1dvOMjcCQ8nP</t>
         </is>
       </c>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
         <is>
           <t>yi_wang_b3MIpYEs1lBUmc9YrTOSQ</t>
         </is>
@@ -1077,14 +1305,26 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>y_y_wang_CaPIAS20yMG27Y6_q-usc</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
-        <v>1</v>
+          <t>['10.1016/j.jad.2021.03.016']</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>['cheung|t', 'jin|y', 'li|w', 'ng|c', 'rao|w', 'xiang|y', 'zhang|q', 'zhao|n', 'zhao|y']</t>
+        </is>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>y_y_wang_CaPIAS20yMG27Y6_q-usc</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1135,14 +1375,26 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>wang_y_-9PvHlx7OaMs2J_Xr9EMJ</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>wang_y_-9PvHlx7OaMs2J_Xr9EMJ</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1193,14 +1445,30 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
+          <t>['10.1140/epjc/s10052-017-4984-5']</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>['University of Virginia']</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
           <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
         </is>
       </c>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+      <c r="R13" t="n">
+        <v>10</v>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1242,7 +1510,11 @@
           <t>wang_y_-JpSGAqJL_fwXDSQFSGML</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>0000-0001-9908-6323</t>
+        </is>
+      </c>
       <c r="K14" t="n">
         <v>1</v>
       </c>
@@ -1251,14 +1523,34 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
+          <t>['10.1093/scan/nsy053']</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>['cai|h', 'gu|r', 'luo|y', 'sedikides|c', 'yang|z']</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>doi:10.1093/scan/nsy053</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>['Institute of Psychology, Chinese Academy of Sciences', 'University of Chinese Academy of Sciences']</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
           <t>wang_y_-JpSGAqJL_fwXDSQFSGML</t>
         </is>
       </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1291,10 +1583,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>wang_y_-PFzUjJUxTfeNfOfUw9P8</t>
@@ -1309,14 +1605,30 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>wang_y_-PFzUjJUxTfeNfOfUw9P8</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep10(2017)072']</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>['Wayne State University']</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>10</v>
+      </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1367,14 +1679,26 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>wang_y_-UUXYgsMgZPLfKnvqQLFU</t>
-        </is>
-      </c>
-      <c r="N16" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevlett.128.122301']</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>wang_y_-UUXYgsMgZPLfKnvqQLFU</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>1</v>
+      </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1416,7 +1740,11 @@
           <t>wang_y_-hemT0OyhC95BtIQ_1OFX</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>0000-0003-3214-4271</t>
+        </is>
+      </c>
       <c r="K17" t="n">
         <v>1</v>
       </c>
@@ -1425,14 +1753,34 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
+          <t>['10.1080/1369118x.2022.2161827']</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>['luo|t']</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>doi:10.1080/1369118x.2022.2161827</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>['Lancaster University', 'London School of Economics and Political Science']</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
           <t>wang_y_-hemT0OyhC95BtIQ_1OFX</t>
         </is>
       </c>
-      <c r="N17" t="n">
-        <v>1</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
+      <c r="R17" t="n">
+        <v>1</v>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1474,7 +1822,11 @@
           <t>wang_y_-lY2eX-UQKRCoijcka_NQ</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>0000-0002-4749-2984</t>
+        </is>
+      </c>
       <c r="K18" t="n">
         <v>1</v>
       </c>
@@ -1483,14 +1835,34 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
+          <t>['10.1051/0004-6361/202346635']</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>doi:10.1051/0004-6361/202346635</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>['Istituto Nazionale di Fisica Nucleare, Sezione di Napoli']</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
           <t>wang_y_-lY2eX-UQKRCoijcka_NQ</t>
         </is>
       </c>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+      <c r="R18" t="n">
+        <v>4</v>
+      </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1541,15 +1913,31 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>wang_y_-p7s7pfG0-xL-_ouFnbPd</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep03(2021)003', '10.1007/jhep12(2021)106']</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
         <is>
+          <t>['Tsinghua University']</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>wang_y_-p7s7pfG0-xL-_ouFnbPd</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>2</v>
+      </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
           <t>wang_y_336A_S8wqdCzUvOQHGyhA</t>
         </is>
       </c>
@@ -1603,14 +1991,26 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>wang_y_-rDCyMD9OASeII_M2g9UN</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep07(2020)116']</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>wang_y_-rDCyMD9OASeII_M2g9UN</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1661,14 +2061,26 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>wang_y_03Ghu9qgEL89Leq7SClAB</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>wang_y_03Ghu9qgEL89Leq7SClAB</t>
+        </is>
+      </c>
+      <c r="R21" t="n">
+        <v>1</v>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1719,14 +2131,26 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>wang_y_03a8RQAWDh8AD6JjVYQVK</t>
-        </is>
-      </c>
-      <c r="N22" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>wang_y_03a8RQAWDh8AD6JjVYQVK</t>
+        </is>
+      </c>
+      <c r="R22" t="n">
+        <v>1</v>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1768,7 +2192,11 @@
           <t>wang_y_05oVTM-N7NdeUtPBLFDfF</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>0000-0002-5902-9399</t>
+        </is>
+      </c>
       <c r="K23" t="n">
         <v>1</v>
       </c>
@@ -1777,14 +2205,34 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
+          <t>['10.1016/j.envsci.2017.05.008']</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>doi:10.1016/j.envsci.2017.05.008</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>["Ministry of Water Resources of the People's Republic of China"]</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
           <t>wang_y_05oVTM-N7NdeUtPBLFDfF</t>
         </is>
       </c>
-      <c r="N23" t="n">
-        <v>1</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
+      <c r="R23" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1826,7 +2274,11 @@
           <t>wang_y_0Fl2lnZ6qcsQSUfbgcnAO</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>0000-0002-0351-3739</t>
+        </is>
+      </c>
       <c r="K24" t="n">
         <v>1</v>
       </c>
@@ -1835,14 +2287,34 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
+          <t>['10.1002/hbm.25364']</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>doi:10.1002/hbm.25364</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>['Medical College of Wisconsin']</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
           <t>wang_y_0Fl2lnZ6qcsQSUfbgcnAO</t>
         </is>
       </c>
-      <c r="N24" t="n">
-        <v>1</v>
-      </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
+      <c r="R24" t="n">
+        <v>1</v>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1875,16 +2347,24 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>wang_y_0H5JjEgPAv2s-7FqSeLPU</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>0000-0002-4749-2984</t>
+        </is>
+      </c>
       <c r="K25" t="n">
         <v>1</v>
       </c>
@@ -1893,14 +2373,30 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>wang_y_0H5JjEgPAv2s-7FqSeLPU</t>
-        </is>
-      </c>
-      <c r="N25" t="n">
-        <v>1</v>
-      </c>
-      <c r="O25" t="inlineStr"/>
+          <t>['10.1051/0004-6361/202141938']</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>doi:10.1051/0004-6361/202141938</t>
+        </is>
+      </c>
       <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>wang_y_-lY2eX-UQKRCoijcka_NQ</t>
+        </is>
+      </c>
+      <c r="R25" t="n">
+        <v>4</v>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1951,14 +2447,26 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>wang_y_0IYQgHkV0k1mreDS4Ma87</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>wang_y_0IYQgHkV0k1mreDS4Ma87</t>
+        </is>
+      </c>
+      <c r="R26" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2009,14 +2517,26 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>wang_y_0OYOhQVadyEcNmCDEbeES</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>1</v>
+          <t>['10.1360/tb-2021-0140']</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>wang_y_0OYOhQVadyEcNmCDEbeES</t>
+        </is>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2067,14 +2587,26 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>wang_y_0WYhoxEBcrKCZ07j74iWs</t>
-        </is>
-      </c>
-      <c r="N28" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.96.032002']</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>wang_y_0WYhoxEBcrKCZ07j74iWs</t>
+        </is>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2107,10 +2639,14 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>wang_y_0_6_p50wCh_JqcEAcOowc</t>
@@ -2125,14 +2661,30 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>wang_y_0_6_p50wCh_JqcEAcOowc</t>
-        </is>
-      </c>
-      <c r="N29" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep04(2019)112', '10.1140/epjc/s10052-016-4573-z']</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>['University of Virginia', 'Wayne State University']</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R29" t="n">
+        <v>10</v>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2165,10 +2717,14 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>wang_y_0fo_af8OrfMgOUCHtICuk</t>
@@ -2183,15 +2739,31 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>wang_y_0fo_af8OrfMgOUCHtICuk</t>
-        </is>
-      </c>
-      <c r="N30" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep02(2018)032']</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
         <is>
+          <t>['Wayne State University']</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R30" t="n">
+        <v>10</v>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
           <t>wang_y_rC5yr7AUokOkt-xONQ4-N</t>
         </is>
       </c>
@@ -2227,10 +2799,14 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>wang_y_0mkmYk-mMPEdpHc7i8DQt</t>
@@ -2245,14 +2821,30 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>wang_y_0mkmYk-mMPEdpHc7i8DQt</t>
-        </is>
-      </c>
-      <c r="N31" t="n">
-        <v>1</v>
+          <t>['10.1140/epjc/s10052-018-6033-4']</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>['University of Virginia']</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R31" t="n">
+        <v>10</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2285,10 +2877,14 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>wang_y_0pCDMrsl2RiBBEhoocHCs</t>
@@ -2303,14 +2899,30 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>wang_y_0pCDMrsl2RiBBEhoocHCs</t>
-        </is>
-      </c>
-      <c r="N32" t="n">
-        <v>1</v>
+          <t>['10.1140/epjc/s10052-016-3988-x']</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>['University of Virginia']</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
+        <v>10</v>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2352,7 +2964,11 @@
           <t>wang_y_0tNAHD3bZxn2Ui7l9S5Ss</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>0009-0006-9208-7538</t>
+        </is>
+      </c>
       <c r="K33" t="n">
         <v>3</v>
       </c>
@@ -2361,18 +2977,38 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
+          <t>['10.1088/1674-1137/44/2/022001', '10.1140/epjc/s10052-020-7733-0']</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>doi:10.1140/epjc/s10052-020-7733-0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>['Central China Normal University']</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
           <t>wang_y_0tNAHD3bZxn2Ui7l9S5Ss</t>
         </is>
       </c>
-      <c r="N33" t="n">
-        <v>1</v>
-      </c>
-      <c r="O33" t="inlineStr">
+      <c r="R33" t="n">
+        <v>2</v>
+      </c>
+      <c r="S33" t="inlineStr">
         <is>
           <t>{'source': "ctx._source.AKA ='wang_y_r77-8yVRKtULJNqfR9nFb'", 'lang': 'painless'}</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2423,14 +3059,30 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
+          <t>['10.1103/physrevb.72.024547']</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>['abe|s', 'filippov|v', 'junod|a', 'lortz|r', 'meingast|c', 'paderno|y']</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>['University of Geneva']</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
           <t>wang_y_0zSWdFwA02iO10F1JcVrK</t>
         </is>
       </c>
-      <c r="N34" t="n">
-        <v>1</v>
-      </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
+      <c r="R34" t="n">
+        <v>3</v>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2463,16 +3115,24 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>wang_y_1KpJitHaSVD9_w_1hzAaK</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>0009-0006-9208-7538</t>
+        </is>
+      </c>
       <c r="K35" t="n">
         <v>1</v>
       </c>
@@ -2481,14 +3141,34 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>wang_y_1KpJitHaSVD9_w_1hzAaK</t>
-        </is>
-      </c>
-      <c r="N35" t="n">
-        <v>1</v>
-      </c>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
+          <t>['10.1103/physrevlett.126.092001']</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>doi:10.1103/physrevlett.126.092001</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>['Central China Normal University']</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>wang_y_0tNAHD3bZxn2Ui7l9S5Ss</t>
+        </is>
+      </c>
+      <c r="R35" t="n">
+        <v>2</v>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2539,14 +3219,26 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>wang_y_1MZfU8pLL3kH7lAnt35sX</t>
-        </is>
-      </c>
-      <c r="N36" t="n">
-        <v>1</v>
+          <t>['10.1140/epjc/s10052-020-08562-y', '10.1140/epjc/s10052-021-08949-5']</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>wang_y_1MZfU8pLL3kH7lAnt35sX</t>
+        </is>
+      </c>
+      <c r="R36" t="n">
+        <v>1</v>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2597,14 +3289,26 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>wang_y_1SR7rLZo_Zw85ClijxR0N</t>
-        </is>
-      </c>
-      <c r="N37" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>['cimiano|p', 'haase|p', 'sure|y', 'völker|j']</t>
+        </is>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>wang_y_1SR7rLZo_Zw85ClijxR0N</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2655,14 +3359,26 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>wang_y_1Y-fHp6ZuVybZ_V6ohBIK</t>
-        </is>
-      </c>
-      <c r="N38" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>wang_y_1Y-fHp6ZuVybZ_V6ohBIK</t>
+        </is>
+      </c>
+      <c r="R38" t="n">
+        <v>1</v>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2713,14 +3429,26 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>wang_y_1fPaYZQflmqRMo_zIZW8l</t>
-        </is>
-      </c>
-      <c r="N39" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevlett.130.211801']</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>wang_y_1fPaYZQflmqRMo_zIZW8l</t>
+        </is>
+      </c>
+      <c r="R39" t="n">
+        <v>1</v>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2753,10 +3481,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>wang_y_1jB46IRMQW4-xe87IfX3d</t>
@@ -2771,14 +3503,30 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>wang_y_1jB46IRMQW4-xe87IfX3d</t>
-        </is>
-      </c>
-      <c r="N40" t="n">
-        <v>1</v>
+          <t>['10.1186/s13102-022-00587-y']</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>['shi|y', 'xiang|l', 'xie|f', 'zhang|j', 'zhang|y']</t>
+        </is>
       </c>
       <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>['Soochow University']</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>wang_y_35gnzflu95nMAzgsH3O2j</t>
+        </is>
+      </c>
+      <c r="R40" t="n">
+        <v>2</v>
+      </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2811,10 +3559,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I41" t="inlineStr">
         <is>
           <t>wang_y_1kLMWg3X0ufiTPAmkTf6u</t>
@@ -2829,14 +3581,30 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>wang_y_1kLMWg3X0ufiTPAmkTf6u</t>
-        </is>
-      </c>
-      <c r="N41" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevb.73.024512']</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>['abe|s', 'junod|a', 'knafo|w', 'lortz|r', 'meingast|c', 'paderno|y', 'popovich|p', 'shitsevalova|n', 'tutsch|u']</t>
+        </is>
       </c>
       <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>['University of Geneva']</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>wang_y_0zSWdFwA02iO10F1JcVrK</t>
+        </is>
+      </c>
+      <c r="R41" t="n">
+        <v>3</v>
+      </c>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2878,7 +3646,11 @@
           <t>wang_y_1qFXoddo4LUvimoP3BzwZ</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>0000-0002-0582-0855</t>
+        </is>
+      </c>
       <c r="K42" t="n">
         <v>1</v>
       </c>
@@ -2887,14 +3659,34 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
+          <t>['10.1088/1361-648x/aaaf3c']</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>['ding|y', 'jiang|y', 'li|z', 'wu|b', 'xu|f', 'yao|y', 'yin|j', 'zhang|p']</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>doi:10.1088/1361-648x/aaaf3c</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>['Fritz Haber Institute of the Max Planck Society']</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
           <t>wang_y_1qFXoddo4LUvimoP3BzwZ</t>
         </is>
       </c>
-      <c r="N42" t="n">
-        <v>1</v>
-      </c>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
+      <c r="R42" t="n">
+        <v>1</v>
+      </c>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2936,7 +3728,11 @@
           <t>wang_y_25-A6xATSJSsdtoUCWchG</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>0000-0001-9831-1090</t>
+        </is>
+      </c>
       <c r="K43" t="n">
         <v>1</v>
       </c>
@@ -2945,14 +3741,34 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
+          <t>['10.1093/cercor/bhab248']</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>doi:10.1093/cercor/bhab248</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>['University of Oslo']</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
           <t>wang_y_25-A6xATSJSsdtoUCWchG</t>
         </is>
       </c>
-      <c r="N43" t="n">
-        <v>1</v>
-      </c>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
+      <c r="R43" t="n">
+        <v>2</v>
+      </c>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2985,10 +3801,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>wang_y_26oPADeoIO2hucrbbqx7r</t>
@@ -3003,14 +3823,30 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>wang_y_26oPADeoIO2hucrbbqx7r</t>
-        </is>
-      </c>
-      <c r="N44" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep12(2017)142']</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>['Wayne State University']</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R44" t="n">
+        <v>10</v>
+      </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3061,14 +3897,26 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>wang_y_2BbSlSFfCeatpAPFkEFnq</t>
-        </is>
-      </c>
-      <c r="N45" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>['bian|l', 'bo|m', 'feng|x', 'guo|j', 'huang|y', 'jiang|c', 'li|z', 'tang|h', 'wei|f', 'xu|x', 'zhang|w', 'zhou|z', 'zou|p', 'zuo|p']</t>
+        </is>
       </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>wang_y_2BbSlSFfCeatpAPFkEFnq</t>
+        </is>
+      </c>
+      <c r="R45" t="n">
+        <v>1</v>
+      </c>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3119,14 +3967,26 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>wang_y_2Cpz7Qtmmo-W_1Z20A3w0</t>
-        </is>
-      </c>
-      <c r="N46" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>wang_y_2Cpz7Qtmmo-W_1Z20A3w0</t>
+        </is>
+      </c>
+      <c r="R46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3177,14 +4037,26 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>wang_y_2KB7wE41Y-gldDEPT02vR</t>
-        </is>
-      </c>
-      <c r="N47" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>wang_y_2KB7wE41Y-gldDEPT02vR</t>
+        </is>
+      </c>
+      <c r="R47" t="n">
+        <v>1</v>
+      </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3226,7 +4098,11 @@
           <t>wang_y_2OxPJdrm6hbzLLJDsWsbO</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>0000-0002-2691-8050</t>
+        </is>
+      </c>
       <c r="K48" t="n">
         <v>1</v>
       </c>
@@ -3235,14 +4111,34 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
+          <t>['10.1093/pm/pnaa148']</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>['du|w', 'guan|x', 'liu|p', 'mao|m', 'ren|y', 'shen|h', 'wei|j', 'zhang|n', 'zhang|y']</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>doi:10.1093/pm/pnaa148</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>['Longhua Hospital Shanghai University of Traditional Chinese Medicine', 'Shanghai University of Traditional Chinese Medicine']</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
           <t>wang_y_2OxPJdrm6hbzLLJDsWsbO</t>
         </is>
       </c>
-      <c r="N48" t="n">
-        <v>1</v>
-      </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
+      <c r="R48" t="n">
+        <v>1</v>
+      </c>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3293,14 +4189,26 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>wang_y_2dGJAqqEz6Cp8pO7l42sv</t>
-        </is>
-      </c>
-      <c r="N49" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.102.112004']</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>wang_y_2dGJAqqEz6Cp8pO7l42sv</t>
+        </is>
+      </c>
+      <c r="R49" t="n">
+        <v>1</v>
+      </c>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3351,14 +4259,26 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>wang_y_2dN-LUR2y4MCguywTWGfF</t>
-        </is>
-      </c>
-      <c r="N50" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>wang_y_2dN-LUR2y4MCguywTWGfF</t>
+        </is>
+      </c>
+      <c r="R50" t="n">
+        <v>1</v>
+      </c>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3400,7 +4320,11 @@
           <t>wang_y_2lD0QZ1Gad18EEGmf2f70</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>0000-0003-2781-8673</t>
+        </is>
+      </c>
       <c r="K51" t="n">
         <v>1</v>
       </c>
@@ -3409,14 +4333,34 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
+          <t>['10.1002/2017jd027199']</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>['ahlgrimm|m', 'bazile|e', 'berg|l', 'cheng|a', 'chéruy|f', 'cole|j', 'forbes|r', 'gustafson|w', 'huang|m', 'klein|s', 'lee|w', 'liu|y', 'ma|h', 'mellul|l', 'merryfield|w', 'morcrette|c', 'petch|j', 'qian|y', 'roehrig|r', 'van weverberg|k', 'xie|s', 'xu|k', 'zhang|c']</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>doi:10.1002/2017jd027199</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>['Academia Sinica']</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
           <t>wang_y_2lD0QZ1Gad18EEGmf2f70</t>
         </is>
       </c>
-      <c r="N51" t="n">
-        <v>1</v>
-      </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr">
+      <c r="R51" t="n">
+        <v>1</v>
+      </c>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
         <is>
           <t>wang_y_As2Q4RvsnrdBUAg8d1qNA</t>
         </is>
@@ -3453,10 +4397,14 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I52" t="inlineStr">
         <is>
           <t>wang_y_31IebXzhDff9dwVAjrRb1</t>
@@ -3471,14 +4419,30 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>wang_y_31IebXzhDff9dwVAjrRb1</t>
-        </is>
-      </c>
-      <c r="N52" t="n">
-        <v>1</v>
+          <t>['10.1140/epjc/s10052-018-5752-x']</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>['University of Virginia']</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R52" t="n">
+        <v>10</v>
+      </c>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3529,14 +4493,26 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>wang_y_31RyZ9qsYmz2ZuH-6wv7t</t>
-        </is>
-      </c>
-      <c r="N53" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>wang_y_31RyZ9qsYmz2ZuH-6wv7t</t>
+        </is>
+      </c>
+      <c r="R53" t="n">
+        <v>1</v>
+      </c>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3578,7 +4554,11 @@
           <t>wang_y_32DTd3qOrAWo4duYpBW6Q</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>0000-0003-1575-0245</t>
+        </is>
+      </c>
       <c r="K54" t="n">
         <v>2</v>
       </c>
@@ -3587,14 +4567,34 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
+          <t>['10.1007/s10796-023-10400-x', '10.1051/0004-6361/202450368']</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>doi:10.1007/s10796-023-10400-x</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>['California Institute of Technology', 'Infrared Processing and Analysis Center', 'University of Sheffield']</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
           <t>wang_y_32DTd3qOrAWo4duYpBW6Q</t>
         </is>
       </c>
-      <c r="N54" t="n">
-        <v>1</v>
-      </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3636,7 +4636,11 @@
           <t>wang_y_35gnzflu95nMAzgsH3O2j</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>0000-0003-1292-0384</t>
+        </is>
+      </c>
       <c r="K55" t="n">
         <v>1</v>
       </c>
@@ -3645,14 +4649,34 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
+          <t>['10.1108/cms-02-2023-0086']</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>['akhtar|m', 'l|y', 'zhang|j', 'zhang|y']</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>doi:10.1108/cms-02-2023-0086</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>['Guangdong University of Foreign Studies']</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
           <t>wang_y_35gnzflu95nMAzgsH3O2j</t>
         </is>
       </c>
-      <c r="N55" t="n">
-        <v>1</v>
-      </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
+      <c r="R55" t="n">
+        <v>2</v>
+      </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3703,14 +4727,26 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>wang_y_3NBuuVkOrQxMjThcqTFgp</t>
-        </is>
-      </c>
-      <c r="N56" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>wang_y_3NBuuVkOrQxMjThcqTFgp</t>
+        </is>
+      </c>
+      <c r="R56" t="n">
+        <v>1</v>
+      </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3761,14 +4797,26 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>wang_y_3PinPOK5UFpdML7v9vdk7</t>
-        </is>
-      </c>
-      <c r="N57" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>wang_y_3PinPOK5UFpdML7v9vdk7</t>
+        </is>
+      </c>
+      <c r="R57" t="n">
+        <v>1</v>
+      </c>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3801,16 +4849,24 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I58" t="inlineStr">
         <is>
           <t>wang_y_3TBI5ZUnTHuZ025IrCbrs</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>0000-0001-9831-1090</t>
+        </is>
+      </c>
       <c r="K58" t="n">
         <v>1</v>
       </c>
@@ -3819,14 +4875,34 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>wang_y_3TBI5ZUnTHuZ025IrCbrs</t>
-        </is>
-      </c>
-      <c r="N58" t="n">
-        <v>1</v>
-      </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
+          <t>['10.5194/isprs-archives-xlvi-m-1-2021-859-2021']</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>['chen|d', 'ma|f', 'wu|x', 'xie|l']</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>doi:10.5194/isprs-archives-xlvi-m-1-2021-859-2021</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>['Central Academy of Fine Arts']</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>wang_y_25-A6xATSJSsdtoUCWchG</t>
+        </is>
+      </c>
+      <c r="R58" t="n">
+        <v>2</v>
+      </c>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3877,14 +4953,26 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>wang_y_3U80BFG9vvD9RFST2i_8B</t>
-        </is>
-      </c>
-      <c r="N59" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>['chen|x', 'gales|m', 'ragni|a', 'wong|j']</t>
+        </is>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>wang_y_3U80BFG9vvD9RFST2i_8B</t>
+        </is>
+      </c>
+      <c r="R59" t="n">
+        <v>1</v>
+      </c>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3926,7 +5014,11 @@
           <t>wang_y_3Vv1J6kx9qo58-h1YN1wj</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>0000-0001-5683-909X</t>
+        </is>
+      </c>
       <c r="K60" t="n">
         <v>1</v>
       </c>
@@ -3935,14 +5027,34 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
+          <t>['10.1098/rsta.2010.0196']</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>['cooper|r', 'e  hussey|n', 'f  xu|x', 'mouzopoulou|i', 'proust|c', 'vignolle|b']</t>
+        </is>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>doi:10.1098/rsta.2010.0196</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>['Peking University', 'University of Bristol']</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
           <t>wang_y_3Vv1J6kx9qo58-h1YN1wj</t>
         </is>
       </c>
-      <c r="N60" t="n">
-        <v>1</v>
-      </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
+      <c r="R60" t="n">
+        <v>1</v>
+      </c>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3984,7 +5096,11 @@
           <t>wang_y_3WVHe_HVm0Gg5wP5FNdtn</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>0000-0003-2499-1147</t>
+        </is>
+      </c>
       <c r="K61" t="n">
         <v>1</v>
       </c>
@@ -3993,14 +5109,34 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
+          <t>['10.5194/cp-12-201-2016']</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>['an|w', 'hou|s', 'liu|y', 'pang|h', 'wu|s', 'zhang|w']</t>
+        </is>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>doi:10.5194/cp-12-201-2016</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>['Shandong Normal University']</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
           <t>wang_y_3WVHe_HVm0Gg5wP5FNdtn</t>
         </is>
       </c>
-      <c r="N61" t="n">
-        <v>1</v>
-      </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
+      <c r="R61" t="n">
+        <v>1</v>
+      </c>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4051,14 +5187,30 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
+          <t>['10.1002/jsfa.1790']</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>['beauchemin|k', 'mcallister|t', 'morgavi|d', 'nsereko|v', 'rode|l']</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>['Agriculture and Agri-Food Canada', 'Lethbridge Research and Development Centre']</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
           <t>wang_y_3Z5RlzyeYcsuZsGFOoAZB</t>
         </is>
       </c>
-      <c r="N62" t="n">
-        <v>1</v>
-      </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
+      <c r="R62" t="n">
+        <v>1</v>
+      </c>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4100,7 +5252,11 @@
           <t>wang_y_3hjII0zNbNtzqNbKefO3O</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>0000-0001-7756-8479</t>
+        </is>
+      </c>
       <c r="K63" t="n">
         <v>1</v>
       </c>
@@ -4109,14 +5265,34 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
+          <t>['10.3847/1538-4365/ab929e']</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>doi:10.3847/1538-4365/ab929e</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>['Chinese Academy of Sciences', 'National Astronomical Observatories']</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
           <t>wang_y_3hjII0zNbNtzqNbKefO3O</t>
         </is>
       </c>
-      <c r="N63" t="n">
-        <v>1</v>
-      </c>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
+      <c r="R63" t="n">
+        <v>2</v>
+      </c>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4167,14 +5343,26 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>wang_y_3o9vODuW0jVQgyczLMc4D</t>
-        </is>
-      </c>
-      <c r="N64" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>wang_y_3o9vODuW0jVQgyczLMc4D</t>
+        </is>
+      </c>
+      <c r="R64" t="n">
+        <v>1</v>
+      </c>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4225,14 +5413,26 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>wang_y_4Dr4t6SEEN0kHIZGhj6V9</t>
-        </is>
-      </c>
-      <c r="N65" t="n">
-        <v>1</v>
+          <t>['10.1016/j.physletb.2021.136188']</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>wang_y_4Dr4t6SEEN0kHIZGhj6V9</t>
+        </is>
+      </c>
+      <c r="R65" t="n">
+        <v>1</v>
+      </c>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4274,7 +5474,11 @@
           <t>wang_y_4KvoOtBm93-pQ67JNSGti</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>0000-0003-3113-7483</t>
+        </is>
+      </c>
       <c r="K66" t="n">
         <v>1</v>
       </c>
@@ -4283,14 +5487,34 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
+          <t>['10.1038/s44304-025-00114-2']</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>['chen|q', 'jiang|h', 'song|d', 'tang|h', 'wei|l']</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>doi:10.1038/s44304-025-00114-2</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>['Lanzhou University of Technology']</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
           <t>wang_y_4KvoOtBm93-pQ67JNSGti</t>
         </is>
       </c>
-      <c r="N66" t="n">
-        <v>1</v>
-      </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
+      <c r="R66" t="n">
+        <v>1</v>
+      </c>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4341,14 +5565,30 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
+          <t>['10.1016/j.physletb.2020.135797']</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>['AGH University of Krakow']</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
           <t>wang_y_4RVTDjzF8bqFDeAkZvBfz</t>
         </is>
       </c>
-      <c r="N67" t="n">
-        <v>1</v>
-      </c>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
+      <c r="R67" t="n">
+        <v>1</v>
+      </c>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4390,7 +5630,11 @@
           <t>wang_y_4T84HfiXUOgxA06Hbv0Ol</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>0000-0002-4614-6203</t>
+        </is>
+      </c>
       <c r="K68" t="n">
         <v>1</v>
       </c>
@@ -4399,14 +5643,34 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
+          <t>['10.5194/bg-6-1341-2009']</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>['carvalhais|n', 'hollinger|d', 'jung|m', 'kattge|j', 'leuning|r', 'luo|y', 'peylin|p', 'reichstein|m', 'richardson|a', 'stoy|p', 'tomelleri|e', 'trudinger|c', 'verbeeck|h', 'williams|m']</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>doi:10.5194/bg-6-1341-2009</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>['CSIRO Oceans and Atmosphere']</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
           <t>wang_y_4T84HfiXUOgxA06Hbv0Ol</t>
         </is>
       </c>
-      <c r="N68" t="n">
-        <v>1</v>
-      </c>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
+      <c r="R68" t="n">
+        <v>1</v>
+      </c>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4439,16 +5703,24 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr">
         <is>
           <t>wang_y_4ncM0CkntTpgdNbvkbTBO</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>0000-0001-7756-8479</t>
+        </is>
+      </c>
       <c r="K69" t="n">
         <v>1</v>
       </c>
@@ -4457,14 +5729,34 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>wang_y_4ncM0CkntTpgdNbvkbTBO</t>
-        </is>
-      </c>
-      <c r="N69" t="n">
-        <v>1</v>
-      </c>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
+          <t>['10.3847/1538-4365/ab929e']</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>doi:10.3847/1538-4365/ab929e</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>['Chinese Academy of Sciences', 'National Astronomical Observatories']</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>wang_y_3hjII0zNbNtzqNbKefO3O</t>
+        </is>
+      </c>
+      <c r="R69" t="n">
+        <v>2</v>
+      </c>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4497,16 +5789,24 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I70" t="inlineStr">
         <is>
           <t>wang_y_4uT8YRQMBZO8hHh6Yhgrz</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>0000-0002-4749-2984</t>
+        </is>
+      </c>
       <c r="K70" t="n">
         <v>1</v>
       </c>
@@ -4515,14 +5815,30 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>wang_y_4uT8YRQMBZO8hHh6Yhgrz</t>
-        </is>
-      </c>
-      <c r="N70" t="n">
-        <v>1</v>
-      </c>
-      <c r="O70" t="inlineStr"/>
+          <t>['10.1051/0004-6361/202141938']</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>doi:10.1051/0004-6361/202141938</t>
+        </is>
+      </c>
       <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>wang_y_-lY2eX-UQKRCoijcka_NQ</t>
+        </is>
+      </c>
+      <c r="R70" t="n">
+        <v>4</v>
+      </c>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4573,14 +5889,30 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
+          <t>['10.1016/j.ajhg.2018.09.009']</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>['Case Western Reserve University', 'QIMR Berghofer Medical Research Institute', 'University Hospitals of Cleveland']</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
           <t>wang_y_5DF-E-tOBaj6AleXkYPtd</t>
         </is>
       </c>
-      <c r="N71" t="n">
-        <v>1</v>
-      </c>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
+      <c r="R71" t="n">
+        <v>1</v>
+      </c>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4631,14 +5963,30 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
+          <t>['10.1016/j.physletb.2016.12.009']</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>['Institute of High Energy Physics']</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
           <t>wang_y_5FUfi-AeIupyPeGGpOar6</t>
         </is>
       </c>
-      <c r="N72" t="n">
-        <v>1</v>
-      </c>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
+      <c r="R72" t="n">
+        <v>1</v>
+      </c>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4671,16 +6019,24 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr">
         <is>
           <t>wang_y_5R2AJyOTKdhQSwgmj5Pl3</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>0000-0002-4749-2984</t>
+        </is>
+      </c>
       <c r="K73" t="n">
         <v>1</v>
       </c>
@@ -4689,14 +6045,34 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>wang_y_5R2AJyOTKdhQSwgmj5Pl3</t>
-        </is>
-      </c>
-      <c r="N73" t="n">
-        <v>1</v>
-      </c>
-      <c r="O73" t="inlineStr"/>
-      <c r="P73" t="inlineStr"/>
+          <t>['10.1051/0004-6361/202556459']</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>doi:10.1051/0004-6361/202556459</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>['California Institute of Technology', 'Infrared Processing and Analysis Center']</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>wang_y_-lY2eX-UQKRCoijcka_NQ</t>
+        </is>
+      </c>
+      <c r="R73" t="n">
+        <v>4</v>
+      </c>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4747,14 +6123,26 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>wang_y_5XoL8NkWi3q0DZCuKg-Df</t>
-        </is>
-      </c>
-      <c r="N74" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>['guo|b', 'lv|q', 'qiu|z', 'zhang|d']</t>
+        </is>
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>wang_y_5XoL8NkWi3q0DZCuKg-Df</t>
+        </is>
+      </c>
+      <c r="R74" t="n">
+        <v>1</v>
+      </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4805,14 +6193,26 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>wang_y_5eZhu_EkRbUXCrSehA-7V</t>
-        </is>
-      </c>
-      <c r="N75" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>wang_y_5eZhu_EkRbUXCrSehA-7V</t>
+        </is>
+      </c>
+      <c r="R75" t="n">
+        <v>1</v>
+      </c>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4845,10 +6245,14 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I76" t="inlineStr">
         <is>
           <t>wang_y_5ivrAdkzsJS5QZC7dLTm5</t>
@@ -4863,14 +6267,30 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>wang_y_5ivrAdkzsJS5QZC7dLTm5</t>
-        </is>
-      </c>
-      <c r="N76" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep10(2021)176']</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr"/>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>['Tsinghua University']</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>wang_y_-p7s7pfG0-xL-_ouFnbPd</t>
+        </is>
+      </c>
+      <c r="R76" t="n">
+        <v>2</v>
+      </c>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4903,10 +6323,14 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr">
         <is>
           <t>wang_y_5vlhi-ZuruJvv1nSI7oY3</t>
@@ -4921,14 +6345,30 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>wang_y_5vlhi-ZuruJvv1nSI7oY3</t>
-        </is>
-      </c>
-      <c r="N77" t="n">
-        <v>1</v>
+          <t>['10.1140/epjc/s10052-017-4828-3']</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O77" t="inlineStr"/>
-      <c r="P77" t="inlineStr"/>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>['University of Virginia']</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R77" t="n">
+        <v>10</v>
+      </c>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4979,14 +6419,26 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>wang_y_6CjMvxqTO2Ak7Kzfzot8g</t>
-        </is>
-      </c>
-      <c r="N78" t="n">
-        <v>1</v>
+          <t>['10.1001/jamapsychiatry.2018.4166']</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>wang_y_6CjMvxqTO2Ak7Kzfzot8g</t>
+        </is>
+      </c>
+      <c r="R78" t="n">
+        <v>1</v>
+      </c>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5037,14 +6489,26 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>wang_y_6D__3dF48bd8I_xUuBFOY</t>
-        </is>
-      </c>
-      <c r="N79" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>wang_y_6D__3dF48bd8I_xUuBFOY</t>
+        </is>
+      </c>
+      <c r="R79" t="n">
+        <v>1</v>
+      </c>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5095,14 +6559,26 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>wang_y_6FOp7XXm0FI1c0fsb_KfB</t>
-        </is>
-      </c>
-      <c r="N80" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep05(2020)052']</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr"/>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>wang_y_6FOp7XXm0FI1c0fsb_KfB</t>
+        </is>
+      </c>
+      <c r="R80" t="n">
+        <v>1</v>
+      </c>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5153,14 +6629,30 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
+          <t>['10.1103/physrevlett.126.122301']</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="O81" t="inlineStr"/>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>['University of Science and Technology of China']</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
           <t>wang_y_6H_1voQVPKEEzlnM4XnO5</t>
         </is>
       </c>
-      <c r="N81" t="n">
-        <v>1</v>
-      </c>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
+      <c r="R81" t="n">
+        <v>1</v>
+      </c>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5202,7 +6694,11 @@
           <t>wang_y_6Wc6UToO3DZZw7tsUdZUv</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>0000-0002-6074-0532</t>
+        </is>
+      </c>
       <c r="K82" t="n">
         <v>1</v>
       </c>
@@ -5211,14 +6707,34 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
+          <t>['10.1007/s11682-016-9649-8']</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>['baker|m', 'baune|b', 'brodaty|h', 'fiatarone singh|m', 'foroughi|n', 'gates|n', 'meiklejohn|j', 'sachdev|p', 'saigal|n', 'singh|n', 'suo|c', 'valenzuela|m', 'wen|w', 'wilson|g']</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>doi:10.1007/s11682-016-9649-8</t>
+        </is>
+      </c>
+      <c r="P82" t="inlineStr">
+        <is>
+          <t>['Hebrew SeniorLife', 'Jean Mayer Human Nutrition Research Center on Aging', 'Tufts University', 'University of California, San Francisco']</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
           <t>wang_y_6Wc6UToO3DZZw7tsUdZUv</t>
         </is>
       </c>
-      <c r="N82" t="n">
-        <v>1</v>
-      </c>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
+      <c r="R82" t="n">
+        <v>2</v>
+      </c>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5269,14 +6785,26 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>wang_y_6cQxjAvbpyzxYG3kRvXvk</t>
-        </is>
-      </c>
-      <c r="N83" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>['chen|h', 'mao|y', 'tang|j', 'wu|z', 'zhou|c']</t>
+        </is>
       </c>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>wang_y_6cQxjAvbpyzxYG3kRvXvk</t>
+        </is>
+      </c>
+      <c r="R83" t="n">
+        <v>1</v>
+      </c>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5327,14 +6855,30 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
+          <t>['10.5194/dwes-1-1-2008']</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>['egli|t', 'hammes|f', 'siebel|e']</t>
+        </is>
+      </c>
+      <c r="O84" t="inlineStr"/>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>['ETH Zurich', 'Institute of Biogeochemistry and Pollutant Dynamics', 'Swiss Federal Institute of Aquatic Science and Technology']</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
           <t>wang_y_6cZH1hQbu9S1JhtV0hH7N</t>
         </is>
       </c>
-      <c r="N84" t="n">
-        <v>1</v>
-      </c>
-      <c r="O84" t="inlineStr"/>
-      <c r="P84" t="inlineStr"/>
+      <c r="R84" t="n">
+        <v>1</v>
+      </c>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5385,14 +6929,26 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>wang_y_6e_uHpxeCuGditV9W1naK</t>
-        </is>
-      </c>
-      <c r="N85" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>['bao|g', 'bartholomot|b', 'craig|p', 'delattre|p', 'giraudoux|p', 'harraga|s', 'quere|j', 'raoul|f', 'shi|d', 'vuitton|d']</t>
+        </is>
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr"/>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>wang_y_6e_uHpxeCuGditV9W1naK</t>
+        </is>
+      </c>
+      <c r="R85" t="n">
+        <v>1</v>
+      </c>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5425,10 +6981,14 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I86" t="inlineStr">
         <is>
           <t>wang_y_6ssmUs0-oYs1lIAEctaUK</t>
@@ -5443,14 +7003,30 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>wang_y_6ssmUs0-oYs1lIAEctaUK</t>
-        </is>
-      </c>
-      <c r="N86" t="n">
-        <v>1</v>
+          <t>['10.1140/epjc/s10052-018-6033-4']</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O86" t="inlineStr"/>
-      <c r="P86" t="inlineStr"/>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>['University of Virginia']</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>wang_y_-IjQ6wu_g-Io2B08xzHM2</t>
+        </is>
+      </c>
+      <c r="R86" t="n">
+        <v>10</v>
+      </c>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5483,16 +7059,24 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t>wang_y_6u7YNTaSJkoC7J8MVEIRv</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>0000-0002-6074-0532</t>
+        </is>
+      </c>
       <c r="K87" t="n">
         <v>1</v>
       </c>
@@ -5501,14 +7085,34 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>wang_y_6u7YNTaSJkoC7J8MVEIRv</t>
-        </is>
-      </c>
-      <c r="N87" t="n">
-        <v>1</v>
-      </c>
-      <c r="O87" t="inlineStr"/>
-      <c r="P87" t="inlineStr"/>
+          <t>['10.1038/mp.2016.19']</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>['baker|m', 'baune|b', 'brodaty|h', 'foroughi|n', 'gates|n', 'lampit|a', 'leung|i', 'mavros|y', 'meiklejohn|j', 'sachdev|p', 'saigal|n', 'singh|m', 'singh|n', 'suo|c', 'valenzuela|m', 'wen|w', 'wilson|g']</t>
+        </is>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>doi:10.1038/mp.2016.19</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>['The University of Sydney', 'University of California, San Francisco']</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>wang_y_6Wc6UToO3DZZw7tsUdZUv</t>
+        </is>
+      </c>
+      <c r="R87" t="n">
+        <v>2</v>
+      </c>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5550,7 +7154,11 @@
           <t>wang_y_79eBI45TyzsERr1Tj1iRQ</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>0000-0003-3360-5842</t>
+        </is>
+      </c>
       <c r="K88" t="n">
         <v>1</v>
       </c>
@@ -5559,14 +7167,34 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
+          <t>['10.5194/isprs-annals-x-3-w1-2022-177-2022']</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>['chen|x']</t>
+        </is>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>doi:10.5194/isprs-annals-x-3-w1-2022-177-2022</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>['China University of Geosciences']</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
           <t>wang_y_79eBI45TyzsERr1Tj1iRQ</t>
         </is>
       </c>
-      <c r="N88" t="n">
-        <v>1</v>
-      </c>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
+      <c r="R88" t="n">
+        <v>1</v>
+      </c>
+      <c r="S88" t="inlineStr"/>
+      <c r="T88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5608,7 +7236,11 @@
           <t>wang_y_7ANYgjke84X7pKev-6hZB</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>0000-0002-5035-0338</t>
+        </is>
+      </c>
       <c r="K89" t="n">
         <v>1</v>
       </c>
@@ -5617,14 +7249,34 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
+          <t>['10.3389/fnhum.2017.00481']</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>['ding|n', 'melloni|l', 'poeppel|d', 'yang|a', 'zhang|w']</t>
+        </is>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>doi:10.3389/fnhum.2017.00481</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>['Zhejiang Gongshang University']</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
           <t>wang_y_7ANYgjke84X7pKev-6hZB</t>
         </is>
       </c>
-      <c r="N89" t="n">
-        <v>1</v>
-      </c>
-      <c r="O89" t="inlineStr"/>
-      <c r="P89" t="inlineStr"/>
+      <c r="R89" t="n">
+        <v>1</v>
+      </c>
+      <c r="S89" t="inlineStr"/>
+      <c r="T89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5657,10 +7309,14 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Wang, Y.</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t>wang_y_7DhOqWO94FOQ-EU9utR36</t>
@@ -5675,14 +7331,30 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>wang_y_7DhOqWO94FOQ-EU9utR36</t>
-        </is>
-      </c>
-      <c r="N90" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevb.72.024547']</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>['abe|s', 'filippov|v', 'junod|a', 'lortz|r', 'meingast|c', 'paderno|y']</t>
+        </is>
       </c>
       <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>['University of Geneva']</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>wang_y_0zSWdFwA02iO10F1JcVrK</t>
+        </is>
+      </c>
+      <c r="R90" t="n">
+        <v>3</v>
+      </c>
+      <c r="S90" t="inlineStr"/>
+      <c r="T90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5733,14 +7405,26 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>wang_y_7MP8M26ZjUoOjGBedlpql</t>
-        </is>
-      </c>
-      <c r="N91" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>['ciblat|p', 'loubaton|p', 'serpedin|e']</t>
+        </is>
       </c>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr"/>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>wang_y_7MP8M26ZjUoOjGBedlpql</t>
+        </is>
+      </c>
+      <c r="R91" t="n">
+        <v>1</v>
+      </c>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5791,14 +7475,26 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>wang_y_v_pX-2_zpE02ssu7i4tjF</t>
-        </is>
-      </c>
-      <c r="N92" t="n">
-        <v>1</v>
+          <t>['10.1038/mp.2016.192']</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr"/>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>wang_y_v_pX-2_zpE02ssu7i4tjF</t>
+        </is>
+      </c>
+      <c r="R92" t="n">
+        <v>1</v>
+      </c>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5849,14 +7545,26 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>wang_y_0Tvu4md-lIbEOGT0YFHg0</t>
-        </is>
-      </c>
-      <c r="N93" t="n">
-        <v>1</v>
+          <t>['10.1051/0004-6361/202038541']</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>['hu|j']</t>
+        </is>
       </c>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr"/>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>wang_y_0Tvu4md-lIbEOGT0YFHg0</t>
+        </is>
+      </c>
+      <c r="R93" t="n">
+        <v>1</v>
+      </c>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5907,14 +7615,26 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>wang_y_5EtHMWvOdiHzOsD8TtXRS</t>
-        </is>
-      </c>
-      <c r="N94" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.104.052008']</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr"/>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>wang_y_5EtHMWvOdiHzOsD8TtXRS</t>
+        </is>
+      </c>
+      <c r="R94" t="n">
+        <v>1</v>
+      </c>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5965,14 +7685,26 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>wang_y_B0aNweTA6Xta36JZ1IxhJ</t>
-        </is>
-      </c>
-      <c r="N95" t="n">
-        <v>1</v>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>['biang|r', 'chang|y', 'dolak|d', 'martino|l', 'patton|t', 'prasad|s', 'quinn|j', 'rosenblatt|d', 'van lonkhuyzen|r', 'vercellone|j', 'yuen|c']</t>
+        </is>
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr"/>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>wang_y_B0aNweTA6Xta36JZ1IxhJ</t>
+        </is>
+      </c>
+      <c r="R95" t="n">
+        <v>1</v>
+      </c>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6023,14 +7755,26 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>wang_y_BDQX0kZR0_9mVcfqMhCsc</t>
-        </is>
-      </c>
-      <c r="N96" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.103.l091102']</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr"/>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>wang_y_BDQX0kZR0_9mVcfqMhCsc</t>
+        </is>
+      </c>
+      <c r="R96" t="n">
+        <v>1</v>
+      </c>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6081,14 +7825,26 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>wang_y_KtQKSc4SNoDpypeSEri8m</t>
-        </is>
-      </c>
-      <c r="N97" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.104.032001']</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr"/>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>wang_y_KtQKSc4SNoDpypeSEri8m</t>
+        </is>
+      </c>
+      <c r="R97" t="n">
+        <v>1</v>
+      </c>
+      <c r="S97" t="inlineStr"/>
+      <c r="T97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6139,14 +7895,26 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>wang_y_RdV6OeURziKY6uqMa2Rdy</t>
-        </is>
-      </c>
-      <c r="N98" t="n">
-        <v>1</v>
+          <t>['10.5194/bg-8-1225-2011']</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>['li|c', 'su|s', 'zhang|y']</t>
+        </is>
       </c>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr"/>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>wang_y_RdV6OeURziKY6uqMa2Rdy</t>
+        </is>
+      </c>
+      <c r="R98" t="n">
+        <v>1</v>
+      </c>
+      <c r="S98" t="inlineStr"/>
+      <c r="T98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6197,14 +7965,26 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>wang_y_zOHzyK9nOouqWMAgQ4D-_</t>
-        </is>
-      </c>
-      <c r="N99" t="n">
-        <v>1</v>
+          <t>['10.1103/physrevd.104.052009']</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr"/>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>wang_y_zOHzyK9nOouqWMAgQ4D-_</t>
+        </is>
+      </c>
+      <c r="R99" t="n">
+        <v>1</v>
+      </c>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6255,14 +8035,26 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>wang_y_8yxRB8cFF4LX7aNmxF_0d</t>
-        </is>
-      </c>
-      <c r="N100" t="n">
-        <v>1</v>
+          <t>['10.1080/00207543.2022.2153942', '10.1080/00207543.2023.2267680']</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>['islam|n', 'jasimuddin|s', 'kamal|m', 'sun|z', 'thomas|a', 'xia|h', 'zhang|j']</t>
+        </is>
       </c>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr"/>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>wang_y_8yxRB8cFF4LX7aNmxF_0d</t>
+        </is>
+      </c>
+      <c r="R100" t="n">
+        <v>1</v>
+      </c>
+      <c r="S100" t="inlineStr"/>
+      <c r="T100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6313,14 +8105,26 @@
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>wang_y_3vEhz_GMMkirtTXC7_E1G</t>
-        </is>
-      </c>
-      <c r="N101" t="n">
-        <v>1</v>
+          <t>['10.1007/jhep07(2023)201', '10.1016/s0140-6736(24)00685-8', '10.29140/jaltcall.v18n1.569']</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>['b|q', 'd|n', 'd|w', 'f|z', 'gy|q', 'g|c', 'g|f', 'h|z', 'j|y', 'k|j', 'k|z', 'm|n', 'm|z', 'q|c', 'q|w', 's|l', 's|t', 'w|h', 'w|z', 'x|l', 'z|r']</t>
+        </is>
       </c>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr"/>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>wang_y_3vEhz_GMMkirtTXC7_E1G</t>
+        </is>
+      </c>
+      <c r="R101" t="n">
+        <v>1</v>
+      </c>
+      <c r="S101" t="inlineStr"/>
+      <c r="T101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>